<commit_message>
Template: students sign in with last name and last 4 code digits
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DBWgAxEPdKsMvJQjwPUR95
</commit_message>
<xml_diff>
--- a/last5/templates/Last5_Import_Template.xlsx
+++ b/last5/templates/Last5_Import_Template.xlsx
@@ -296,7 +296,7 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Required. Students sign in with their last name and 8-digit code.</t>
+        <t>Required. Students sign in with their last name and the last 4 digits of their code.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Required. Students sign in with their last name and 8-digit code.</t>
+          <t>Required. Students sign in with their last name and the last 4 digits of their code.</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">

</xml_diff>